<commit_message>
Publish HSK1 vocabulary files 8, 9, and 10 to external repository - Added binary content for HSK1_parts_of_speech_10(451-500).xlsx - Updated metadata for HSK1_parts_of_speech_9(401-450).xlsx - Verified publication status via file size and timestamp checks
</commit_message>
<xml_diff>
--- a/HSK1_parts_of_speech_10(451-500).xlsx
+++ b/HSK1_parts_of_speech_10(451-500).xlsx
@@ -601,6 +601,21 @@
           <t>далёкий</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>дальность (远近)</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>далёкий</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>далеко (离得远)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -627,6 +642,16 @@
           <t>месяц</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>месяц; луна</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>для месяцев (一个月)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -653,6 +678,11 @@
           <t>снова</t>
         </is>
       </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>снова, ещё раз; потом (先…再… — сначала…, а потом…)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -679,6 +709,16 @@
           <t>до свидания</t>
         </is>
       </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>до свидания!</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>устойчивое прощальное выражение</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -705,6 +745,21 @@
           <t>находиться в...</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>находиться (в/на/у); существовать</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>в процессе (在 + V: 在看书 — читает сейчас)</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>в, на (在 + место: 在家 — дома)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -731,6 +786,16 @@
           <t>дома</t>
         </is>
       </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>дома (находиться дома)</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>словосочетание: предлог 在 + существительное 家</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -757,6 +822,21 @@
           <t>утро; ранний</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>утро; ранний час</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>ранний</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>рано (起得早)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -783,6 +863,11 @@
           <t>завтрак</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>завтрак</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -809,6 +894,11 @@
           <t>утро</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>утро (早上 = раннее время дня)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -835,6 +925,21 @@
           <t>каким образом</t>
         </is>
       </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>как, каким образом (疑问代词)</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>почему, как так (怎么不来说 — почему же не пришёл)</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>ну как же! (怎么会!)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -861,6 +966,21 @@
           <t>стоять</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>станция, остановка</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>стоять</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>для станций/стоянок (一站路 — один перегон пешком)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -887,6 +1007,11 @@
           <t>искать</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>искать, разыскивать</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -913,6 +1038,16 @@
           <t>найти</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>найти, отыскать</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>глагол + результативное дополнение 到 (结果补语)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -939,6 +1074,16 @@
           <t>этот</t>
         </is>
       </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>этот, это (这里/这些)</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>этот (这 + счётное слово: 这个人 — этот человек)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -965,6 +1110,16 @@
           <t>здесь, в этих местах</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>эта сторона, здесь</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>здесь, в этих краях</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -991,6 +1146,11 @@
           <t>здесь</t>
         </is>
       </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>здесь, тут (это место)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1017,6 +1177,11 @@
           <t>здесь</t>
         </is>
       </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>здесь, тут (разговорная форма 这里)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1043,6 +1208,11 @@
           <t>эти</t>
         </is>
       </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>эти (множественное от 这)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1069,6 +1239,21 @@
           <t>показатель длительности действия или состояния</t>
         </is>
       </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>частица длительности/продолженного состояния (V + 着)</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>служебная часть речи, самостоятельного значения не имеет</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>Самостоятельно не употребляется</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1095,6 +1280,26 @@
           <t>действительный</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>истина (真相)</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>настоящий, подлинный</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>действительно, в самом деле (真好 — правда хорошо)</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>подлинный (真皮 — натуральная кожа)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1121,6 +1326,21 @@
           <t>действительный; действительно</t>
         </is>
       </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>настоящий, искренний</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>действительно, вправду</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>усилительная конструкция</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1147,6 +1367,26 @@
           <t>прямо, точно</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>правильность (立正 — смирно!)</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>правильный, ровный (正 = 正确)</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>как раз, ровно (正好); прямо (正中间)</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>правильный, основной (正月 — первый лунный месяц)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1173,6 +1413,16 @@
           <t>быть в процессе...</t>
         </is>
       </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>как раз сейчас, в процессе (正在 + V)</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>грамматическая конструкция продолженного действия</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1199,6 +1449,11 @@
           <t>знать</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>знать, осознавать</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1225,6 +1480,11 @@
           <t>знания</t>
         </is>
       </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>знание, знания</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1251,6 +1511,21 @@
           <t>центр; центральный</t>
         </is>
       </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>середина, центр</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>китайский (только в составе: 中国, 中文)</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>средний, внутри (中年 — средних лет; 水中 — в воде)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1277,6 +1552,11 @@
           <t>Китай</t>
         </is>
       </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Китай</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1303,6 +1583,11 @@
           <t>посередине</t>
         </is>
       </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>середина, середина чего-л.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1329,6 +1614,11 @@
           <t>китайский язык</t>
         </is>
       </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>китайский язык (письменный/устный)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1355,6 +1645,11 @@
           <t>полдень</t>
         </is>
       </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>полдень, обеденное время</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1381,6 +1676,11 @@
           <t>средняя школа</t>
         </is>
       </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>средняя школа</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1407,6 +1707,11 @@
           <t>ученик средней школы</t>
         </is>
       </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>ученик средней школы</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1433,6 +1738,26 @@
           <t>тяжёлый</t>
         </is>
       </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>вес (多重多少)</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>повторять (chóng: 重复)</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>тяжёлый (体重); важный</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>тяжело (说话很重 — говорить резко)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1459,6 +1784,11 @@
           <t>важный</t>
         </is>
       </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>важный</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1485,6 +1815,11 @@
           <t>жить</t>
         </is>
       </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>жить, проживать; поселиться</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1511,6 +1846,26 @@
           <t>быть готовым</t>
         </is>
       </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>подготовка (в составе: 准备工作)</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>готовить, подготавливаться</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>приблизительно, примерно (准备三天 — около трёх дней)</t>
+        </is>
+      </c>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>离合词: 准备好了</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1542,6 +1897,11 @@
           <t>да</t>
         </is>
       </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>стол</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1568,6 +1928,16 @@
           <t>иероглиф</t>
         </is>
       </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>иероглиф, знак; письмо, почерк (写字)</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>для иероглифов/надписей (一个字)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1604,6 +1974,21 @@
           <t>нет</t>
         </is>
       </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>суффикс существительных (桌子, 孩子, 儿子)</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>словообразовательный суффикс, самостоятельная единица только в составе слов</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>Самостоятельно не употребляется</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1630,6 +2015,11 @@
           <t>ходить, идти</t>
         </is>
       </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>идти, ходить; уходить</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1656,6 +2046,16 @@
           <t>ходить пешком</t>
         </is>
       </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>ходить пешком</t>
+        </is>
+      </c>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t>离合词: 走了一段路</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1682,6 +2082,11 @@
           <t>самый</t>
         </is>
       </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>самый, наиболее (最 + прилаг.)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1708,6 +2113,16 @@
           <t>лучший</t>
         </is>
       </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>лучше всего, желательно (你最好去 — тебе лучше пойти)</t>
+        </is>
+      </c>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>устойчивое сочетание 最 + 好</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1734,6 +2149,21 @@
           <t>последний</t>
         </is>
       </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>конец, финал (到最后 — до конца)</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>в конце концов, наконец</t>
+        </is>
+      </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>последний, итоговый (最后一步 — последний шаг)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1760,6 +2190,21 @@
           <t>вчера</t>
         </is>
       </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>вчера (время)</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>вчера</t>
+        </is>
+      </c>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>вчерашний (昨天的事)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1786,6 +2231,21 @@
           <t>левый</t>
         </is>
       </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>левая сторона</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>левый</t>
+        </is>
+      </c>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>левый (左手)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1812,6 +2272,11 @@
           <t>слева, левая сторона</t>
         </is>
       </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>слева, левая сторона</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1838,6 +2303,16 @@
           <t>сидеть</t>
         </is>
       </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>сидеть; ездить (坐飞机 — лететь самолётом)</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>на, посредством (坐 + транспорт)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1864,6 +2339,16 @@
           <t>сесть</t>
         </is>
       </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>сесть, садиться</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>глагол + направленное дополнение 下 (趋向补语)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1888,6 +2373,11 @@
       <c r="I51" t="inlineStr">
         <is>
           <t>делать</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>делать; изготавливать (做饭)</t>
         </is>
       </c>
     </row>

</xml_diff>